<commit_message>
chore: updates to output templates to reflect Q1_2026 instead of Q4_2025
</commit_message>
<xml_diff>
--- a/packages/server/src/arpa_reporter/data/treasury/project18_229233BulkUpload.xlsx
+++ b/packages/server/src/arpa_reporter/data/treasury/project18_229233BulkUpload.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kgu82\Desktop\SLFRFBulkUploadTemplates\SLFRFBulkUploadTemplates\SLFRFBulkUploadTemplates\SLFRFBulkUploadTemplates\Quarter 4 2025 Project Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Mac\Home\Documents\Projects\arpa-reporter\packages\server\src\arpa_reporter\data\treasury\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930754BE-1696-4F65-8533-D549D490875E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64C8E55C-89BA-4D38-9F9E-EB1D9243BF76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1270" yWindow="890" windowWidth="25580" windowHeight="15420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -483,10 +483,10 @@
     <t>This project earned program income</t>
   </si>
   <si>
-    <t>Q4_2025_Obligations__c</t>
+    <t>Q1_2026_Obligations__c</t>
   </si>
   <si>
-    <t>Q4_2025_Expenditures__c</t>
+    <t>Q1_2026_Expenditures__c</t>
   </si>
 </sst>
 </file>
@@ -871,14 +871,14 @@
     <col min="1" max="1" width="53" style="3" customWidth="1"/>
     <col min="2" max="20" width="35.5" style="3" customWidth="1"/>
     <col min="21" max="21" width="29" style="3" customWidth="1"/>
-    <col min="22" max="25" width="25.09765625" style="3" customWidth="1"/>
-    <col min="26" max="26" width="28.8984375" style="3" customWidth="1"/>
-    <col min="27" max="28" width="29.8984375" style="3" customWidth="1"/>
-    <col min="29" max="36" width="25.59765625" style="3" customWidth="1"/>
+    <col min="22" max="25" width="25.08203125" style="3" customWidth="1"/>
+    <col min="26" max="26" width="28.9140625" style="3" customWidth="1"/>
+    <col min="27" max="28" width="29.9140625" style="3" customWidth="1"/>
+    <col min="29" max="36" width="25.58203125" style="3" customWidth="1"/>
     <col min="37" max="16384" width="12.5" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>83</v>
       </c>
@@ -918,7 +918,7 @@
       <c r="AI1" s="2"/>
       <c r="AJ1" s="2"/>
     </row>
-    <row r="2" spans="1:36" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" ht="25" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>51</v>
       </c>
@@ -998,7 +998,7 @@
       <c r="AI3" s="2"/>
       <c r="AJ3" s="2"/>
     </row>
-    <row r="4" spans="1:36" ht="66.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" ht="66.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>0</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="5" spans="1:36" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>16</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:36" ht="52.8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" ht="50" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>30</v>
       </c>
@@ -1328,7 +1328,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:36" ht="409.6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>18</v>
       </c>
@@ -1438,7 +1438,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:36" ht="43.35" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" ht="43.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -1476,7 +1476,7 @@
       <c r="AI8" s="2"/>
       <c r="AJ8" s="2"/>
     </row>
-    <row r="9" spans="1:36" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -1514,7 +1514,7 @@
       <c r="AI9" s="2"/>
       <c r="AJ9" s="2"/>
     </row>
-    <row r="10" spans="1:36" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1552,7 +1552,7 @@
       <c r="AI10" s="2"/>
       <c r="AJ10" s="2"/>
     </row>
-    <row r="11" spans="1:36" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -1590,7 +1590,7 @@
       <c r="AI11" s="2"/>
       <c r="AJ11" s="2"/>
     </row>
-    <row r="12" spans="1:36" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -1628,7 +1628,7 @@
       <c r="AI12" s="2"/>
       <c r="AJ12" s="2"/>
     </row>
-    <row r="13" spans="1:36" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -1666,7 +1666,7 @@
       <c r="AI13" s="2"/>
       <c r="AJ13" s="2"/>
     </row>
-    <row r="14" spans="1:36" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -1704,7 +1704,7 @@
       <c r="AI14" s="2"/>
       <c r="AJ14" s="2"/>
     </row>
-    <row r="15" spans="1:36" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -1742,7 +1742,7 @@
       <c r="AI15" s="2"/>
       <c r="AJ15" s="2"/>
     </row>
-    <row r="16" spans="1:36" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:36" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -1780,7 +1780,7 @@
       <c r="AI16" s="2"/>
       <c r="AJ16" s="2"/>
     </row>
-    <row r="17" spans="1:36" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -1818,7 +1818,7 @@
       <c r="AI17" s="2"/>
       <c r="AJ17" s="2"/>
     </row>
-    <row r="18" spans="1:36" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:36" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -1856,7 +1856,7 @@
       <c r="AI18" s="2"/>
       <c r="AJ18" s="2"/>
     </row>
-    <row r="19" spans="1:36" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:36" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -1894,7 +1894,7 @@
       <c r="AI19" s="2"/>
       <c r="AJ19" s="2"/>
     </row>
-    <row r="20" spans="1:36" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:36" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -39174,15 +39174,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FD7D29C8E3DCB740B512085BDB890A19" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="252040482c07e84078604bad08e1f478">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1998147e-1bae-4425-a5b5-824e2b69f76d" xmlns:ns3="79f0e6e4-ac4e-4584-83f0-2cc69c4e4aae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a426bac492543af192e091bebadc75c6" ns2:_="" ns3:_="">
     <xsd:import namespace="1998147e-1bae-4425-a5b5-824e2b69f76d"/>
@@ -39399,6 +39390,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -39406,14 +39406,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D55B629F-9BAD-43E6-819F-B097A47F8C05}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6D20EFE-128A-4BEA-B77D-8F21601543E1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -39428,6 +39420,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D55B629F-9BAD-43E6-819F-B097A47F8C05}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>